<commit_message>
Standardize extracted invoice dates
</commit_message>
<xml_diff>
--- a/outputs/invoice_summary.xlsx
+++ b/outputs/invoice_summary.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>23.05.2021</t>
+          <t>2021-05-23</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -521,12 +521,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>24.06.2020</t>
+          <t>2020-06-24</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>24.09.2020</t>
+          <t>2020-09-24</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
@@ -543,12 +543,12 @@
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
-          <t>October 12, 2021</t>
+          <t>2021-10-12</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>November 12, 2021</t>
+          <t>2021-11-12</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -585,12 +585,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>27.08.2019</t>
+          <t>2019-08-27</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>27.09.2019</t>
+          <t>2019-09-27</t>
         </is>
       </c>
       <c r="E5" t="inlineStr"/>
@@ -611,7 +611,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>16.12.2021</t>
+          <t>2021-12-16</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>

</xml_diff>

<commit_message>
Clean console output and improve batch processing summary
</commit_message>
<xml_diff>
--- a/outputs/invoice_summary.xlsx
+++ b/outputs/invoice_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,21 @@
           <t>total_due</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>missing_core_fields</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>missing_optional_fields</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -505,6 +520,17 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>6610.95</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>due_date</t>
         </is>
       </c>
     </row>
@@ -533,6 +559,21 @@
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>REVIEW NEEDED</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>total_due</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>subtotal, sales_tax, shipping_handling</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -571,6 +612,17 @@
           <t>213470</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>REVIEW NEEDED</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>invoice_number</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -597,6 +649,21 @@
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>REVIEW NEEDED</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>total_due</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>subtotal, sales_tax, shipping_handling</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -629,6 +696,17 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>2809.30</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>OK</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>due_date, shipping_handling</t>
         </is>
       </c>
     </row>

</xml_diff>